<commit_message>
Phase 2: Power Query refinement layer (FACT_TACS_Matching + source loaders)
Injects realistic overlap between FACT_Asset and FACT_Host into the mock
data (previously disjoint, which made any matching logic trivially
NO_MATCH-only), scoped FACT_TACS_Matching to Asset-grain (100 rows) instead
of the plan's literal 500 since the join is asset-to-host by nature.

Adds M query code for all five source loaders plus the two-pass
(장비명=호스트명 -> 장비IP=대표IP) matching logic, parameterized via
SourceFolder for a later real-data swap. Validated against mock data in
Python: MATCH 80% / NAME_MATCH 5% / IP_MATCH 5% / NO_MATCH 10%, matching
the plan's target distribution exactly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mock-data/out/장비 목록_무선_20260828.xlsx
+++ b/mock-data/out/장비 목록_무선_20260828.xlsx
@@ -524,7 +524,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ASSET0071</t>
+          <t>ASSET0092</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -539,12 +539,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KT-WBR-GWANGJU-01</t>
+          <t>KTAI040</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>10.10.1.241</t>
+          <t>10.24.1.252</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -554,17 +554,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Wireless-Bridge</t>
+          <t>WLC</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>개발</t>
+          <t>운영</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>IDC운용팀</t>
+          <t>NW운용2팀</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -589,24 +589,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NTP-GROUP-02</t>
+          <t>NTP-GROUP-01</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>GWANGJU IDC Wireless-Bridge</t>
+          <t>GWANGJU IDC WLC</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R2" s="1" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -614,13 +614,13 @@
         </is>
       </c>
       <c r="T2" s="1" t="n">
-        <v>45296</v>
+        <v>45368</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ASSET0072</t>
+          <t>ASSET0089</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -630,17 +630,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>인프라부문</t>
+          <t>네트워크부문</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KT-WLC-SEOUL-02</t>
+          <t>KTAI023</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>10.10.1.7</t>
+          <t>10.24.1.128</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -655,12 +655,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>운영</t>
+          <t>개발</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>IDC운용팀</t>
+          <t>Cloud사업팀</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -690,33 +690,33 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>NTP-GROUP-02</t>
+          <t>NTP-GROUP-03</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>SEOUL IDC WLC</t>
+          <t>INCHEON IDC WLC</t>
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="R3" s="1" t="n">
-        <v>46252</v>
+        <v>46261</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>자동</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="T3" s="1" t="n">
-        <v>45692</v>
+        <v>45669</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ASSET0073</t>
+          <t>ASSET0085</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -726,17 +726,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>네트워크부문</t>
+          <t>인프라부문</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KT-AP-INCHEON-03</t>
+          <t>KTIPTV052</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.10.13.213</t>
+          <t>10.22.2.38</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>Wireless-Bridge</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>미적용</t>
+          <t>적용</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -791,14 +791,14 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>INCHEON IDC AP</t>
+          <t>BUSAN IDC Wireless-Bridge</t>
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="R4" s="1" t="n">
-        <v>46234</v>
+        <v>46262</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -806,13 +806,13 @@
         </is>
       </c>
       <c r="T4" s="1" t="n">
-        <v>45739</v>
+        <v>45342</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ASSET0074</t>
+          <t>ASSET0098</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -827,12 +827,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KT-AP-SEOUL-04</t>
+          <t>KTIPTV061</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.10.5.130</t>
+          <t>10.22.2.96</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -842,17 +842,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>WLC</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>개발</t>
+          <t>운영</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NW운용2팀</t>
+          <t>Cloud사업팀</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>미적용</t>
+          <t>적용</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -882,19 +882,19 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>NTP-GROUP-01</t>
+          <t>NTP-GROUP-03</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>SEOUL IDC AP</t>
+          <t>BUSAN IDC WLC</t>
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="R5" s="1" t="n">
-        <v>46257</v>
+        <v>46252</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -902,13 +902,13 @@
         </is>
       </c>
       <c r="T5" s="1" t="n">
-        <v>45303</v>
+        <v>45502</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASSET0075</t>
+          <t>ASSET0084</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -918,17 +918,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>보안부문</t>
+          <t>네트워크부문</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KT-WBR-INCHEON-05</t>
+          <t>KTGE023</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>10.10.5.8</t>
+          <t>10.23.1.118</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Wireless-Bridge</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>PAN-OS</t>
+          <t>IOS-XE</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>12.5</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>적용</t>
+          <t>미적용</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -978,19 +978,19 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>NTP-GROUP-01</t>
+          <t>NTP-GROUP-02</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>INCHEON IDC Wireless-Bridge</t>
+          <t>DAEJEON IDC AP</t>
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R6" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -998,13 +998,13 @@
         </is>
       </c>
       <c r="T6" s="1" t="n">
-        <v>45840</v>
+        <v>45509</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ASSET0076</t>
+          <t>ASSET0080</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>인프라부문</t>
+          <t>보안부문</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KT-AP-GWANGJU-06</t>
+          <t>KTAI015</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>10.10.9.169</t>
+          <t>10.24.1.87</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>NW운용1팀</t>
+          <t>NW운용2팀</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1064,22 +1064,22 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>적용</t>
+          <t>미적용</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>NTP-GROUP-01</t>
+          <t>NTP-GROUP-03</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>GWANGJU IDC AP</t>
+          <t>SEOUL IDC AP</t>
         </is>
       </c>
       <c r="Q7" t="n">
@@ -1094,13 +1094,13 @@
         </is>
       </c>
       <c r="T7" s="1" t="n">
-        <v>45581</v>
+        <v>45770</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ASSET0077</t>
+          <t>ASSET0082</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1110,17 +1110,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>보안부문</t>
+          <t>인프라부문</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KT-WLC-BUSAN-07</t>
+          <t>KTBCP012</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>10.10.3.20</t>
+          <t>10.25.1.53</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>NW운용1팀</t>
+          <t>NW운용2팀</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1175,14 +1175,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>BUSAN IDC WLC</t>
+          <t>GWANGJU IDC WLC</t>
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1190,13 +1190,13 @@
         </is>
       </c>
       <c r="T8" s="1" t="n">
-        <v>45995</v>
+        <v>45752</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ASSET0078</t>
+          <t>ASSET0083</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1206,17 +1206,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>인프라부문</t>
+          <t>보안부문</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KT-WLC-GWANGJU-08</t>
+          <t>KTDB062</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>10.10.11.163</t>
+          <t>10.21.2.159</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>WLC</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1241,17 +1241,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Network OS</t>
+          <t>Linux</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>IOS-XE</t>
+          <t>Rocky Linux</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>13.4</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1266,19 +1266,19 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>NTP-GROUP-02</t>
+          <t>NTP-GROUP-01</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>GWANGJU IDC WLC</t>
+          <t>SEOUL IDC AP</t>
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="R9" s="1" t="n">
-        <v>46261</v>
+        <v>46252</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1286,13 +1286,13 @@
         </is>
       </c>
       <c r="T9" s="1" t="n">
-        <v>45920</v>
+        <v>45366</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ASSET0079</t>
+          <t>ASSET0093</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1307,12 +1307,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KT-WBR-INCHEON-09</t>
+          <t>KTDB058</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>10.10.1.41</t>
+          <t>10.21.2.124</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Wireless-Bridge</t>
+          <t>WLC</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1332,22 +1332,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>NW운용1팀</t>
+          <t>IDC운용팀</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Linux</t>
+          <t>Network OS</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Rocky Linux</t>
+          <t>JunOS</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1362,19 +1362,19 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>NTP-GROUP-01</t>
+          <t>NTP-GROUP-02</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>INCHEON IDC Wireless-Bridge</t>
+          <t>SEOUL IDC WLC</t>
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R10" s="1" t="n">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1382,13 +1382,13 @@
         </is>
       </c>
       <c r="T10" s="1" t="n">
-        <v>45409</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ASSET0080</t>
+          <t>ASSET0077</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1403,12 +1403,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KT-AP-SEOUL-10</t>
+          <t>KTCLD023</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>10.10.11.36</t>
+          <t>10.20.1.173</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>WLC</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NW운용2팀</t>
+          <t>NW운용1팀</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>미적용</t>
+          <t>적용</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>SEOUL IDC AP</t>
+          <t>BUSAN IDC WLC</t>
         </is>
       </c>
       <c r="Q11" t="n">
@@ -1478,13 +1478,13 @@
         </is>
       </c>
       <c r="T11" s="1" t="n">
-        <v>45770</v>
+        <v>45995</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ASSET0081</t>
+          <t>ASSET0100</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1494,17 +1494,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>보안부문</t>
+          <t>인프라부문</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KT-WBR-GWANGJU-11</t>
+          <t>KTIPTV044</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10.10.14.132</t>
+          <t>10.22.1.253</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1529,17 +1529,17 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Network OS</t>
+          <t>Linux</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>IOS-XE</t>
+          <t>Rocky Linux</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1549,24 +1549,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>NTP-GROUP-03</t>
+          <t>NTP-GROUP-01</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>GWANGJU IDC Wireless-Bridge</t>
+          <t>SEOUL IDC Wireless-Bridge</t>
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R12" s="1" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1574,13 +1574,13 @@
         </is>
       </c>
       <c r="T12" s="1" t="n">
-        <v>46196</v>
+        <v>46070</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ASSET0082</t>
+          <t>ASSET0094</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1590,17 +1590,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>인프라부문</t>
+          <t>네트워크부문</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KT-WLC-GWANGJU-12</t>
+          <t>KTCLD066</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.10.20.192</t>
+          <t>10.20.2.217</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>WLC</t>
+          <t>Wireless-Bridge</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1620,22 +1620,22 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>NW운용2팀</t>
+          <t>Cloud사업팀</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Linux</t>
+          <t>Network OS</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Rocky Linux</t>
+          <t>JunOS</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>15.9</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1655,14 +1655,14 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>GWANGJU IDC WLC</t>
+          <t>SEOUL IDC Wireless-Bridge</t>
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R13" s="1" t="n">
-        <v>46262</v>
+        <v>46257</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1670,13 +1670,13 @@
         </is>
       </c>
       <c r="T13" s="1" t="n">
-        <v>45752</v>
+        <v>45442</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ASSET0083</t>
+          <t>ASSET0090</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>KT-AP-SEOUL-13</t>
+          <t>KTBCP055</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>10.10.17.65</t>
+          <t>10.25.2.27</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>Wireless-Bridge</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1716,22 +1716,22 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>NW운용1팀</t>
+          <t>Cloud사업팀</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Linux</t>
+          <t>Network OS</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Rocky Linux</t>
+          <t>IOS-XE</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1751,14 +1751,14 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>SEOUL IDC AP</t>
+          <t>SEOUL IDC Wireless-Bridge</t>
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="R14" s="1" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1766,13 +1766,13 @@
         </is>
       </c>
       <c r="T14" s="1" t="n">
-        <v>45366</v>
+        <v>45414</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ASSET0084</t>
+          <t>ASSET0088</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1782,17 +1782,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>네트워크부문</t>
+          <t>인프라부문</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>KT-AP-DAEJEON-14</t>
+          <t>KTGE065</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.10.12.38</t>
+          <t>10.23.2.87</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>WLC</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1822,17 +1822,17 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>IOS-XE</t>
+          <t>JunOS</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>12.8</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>미적용</t>
+          <t>적용</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1842,33 +1842,33 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>NTP-GROUP-02</t>
+          <t>NTP-GROUP-03</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>DAEJEON IDC AP</t>
+          <t>DAEJEON IDC WLC</t>
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R15" s="1" t="n">
-        <v>46260</v>
+        <v>46257</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>자동</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="T15" s="1" t="n">
-        <v>45509</v>
+        <v>45416</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ASSET0085</t>
+          <t>ASSET0091</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1883,12 +1883,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KT-WBR-BUSAN-15</t>
+          <t>KTCLD012</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>10.10.4.144</t>
+          <t>10.20.1.131</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1898,17 +1898,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Wireless-Bridge</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>개발</t>
+          <t>운영</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Cloud사업팀</t>
+          <t>NW운용1팀</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1943,14 +1943,14 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>BUSAN IDC Wireless-Bridge</t>
+          <t>DAEJEON IDC AP</t>
         </is>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R16" s="1" t="n">
-        <v>46262</v>
+        <v>46257</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -1958,13 +1958,13 @@
         </is>
       </c>
       <c r="T16" s="1" t="n">
-        <v>45342</v>
+        <v>45579</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ASSET0086</t>
+          <t>ASSET0081</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1974,17 +1974,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>네트워크부문</t>
+          <t>보안부문</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KT-WLC-GWANGJU-16</t>
+          <t>KTGE043</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>10.10.2.254</t>
+          <t>10.23.1.236</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>WLC</t>
+          <t>Wireless-Bridge</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2004,22 +2004,22 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Cloud사업팀</t>
+          <t>IDC운용팀</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Linux</t>
+          <t>Network OS</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Rocky Linux</t>
+          <t>IOS-XE</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>14.2</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2034,19 +2034,19 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>NTP-GROUP-01</t>
+          <t>NTP-GROUP-03</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>GWANGJU IDC WLC</t>
+          <t>GWANGJU IDC Wireless-Bridge</t>
         </is>
       </c>
       <c r="Q17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R17" s="1" t="n">
-        <v>46257</v>
+        <v>46260</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -2054,13 +2054,13 @@
         </is>
       </c>
       <c r="T17" s="1" t="n">
-        <v>46168</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ASSET0087</t>
+          <t>ASSET0095</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2070,17 +2070,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>인프라부문</t>
+          <t>네트워크부문</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>KT-WBR-SEOUL-17</t>
+          <t>KTGE034</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>10.10.15.73</t>
+          <t>10.23.1.172</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2090,17 +2090,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Wireless-Bridge</t>
+          <t>WLC</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>개발</t>
+          <t>운영</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>NW운용1팀</t>
+          <t>Cloud사업팀</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2130,19 +2130,19 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>NTP-GROUP-02</t>
+          <t>NTP-GROUP-03</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>SEOUL IDC Wireless-Bridge</t>
+          <t>SEOUL IDC WLC</t>
         </is>
       </c>
       <c r="Q18" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="R18" s="1" t="n">
-        <v>46246</v>
+        <v>46260</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -2150,13 +2150,13 @@
         </is>
       </c>
       <c r="T18" s="1" t="n">
-        <v>46113</v>
+        <v>45733</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ASSET0088</t>
+          <t>ASSET0099</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2166,17 +2166,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>인프라부문</t>
+          <t>네트워크부문</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>KT-WLC-DAEJEON-18</t>
+          <t>KTGE050</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>10.10.9.82</t>
+          <t>10.23.2.13</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>WLC</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2196,22 +2196,22 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>IDC운용팀</t>
+          <t>Cloud사업팀</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Network OS</t>
+          <t>Linux</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>JunOS</t>
+          <t>Rocky Linux</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>12.8</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2231,28 +2231,28 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>DAEJEON IDC WLC</t>
+          <t>BUSAN IDC AP</t>
         </is>
       </c>
       <c r="Q19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R19" s="1" t="n">
-        <v>46257</v>
+        <v>46262</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>자동</t>
         </is>
       </c>
       <c r="T19" s="1" t="n">
-        <v>45416</v>
+        <v>45614</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ASSET0089</t>
+          <t>ASSET0071</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2262,17 +2262,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>네트워크부문</t>
+          <t>보안부문</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KT-WLC-INCHEON-19</t>
+          <t>KTAI074</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.10.4.8</t>
+          <t>10.24.2.209</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>WLC</t>
+          <t>Wireless-Bridge</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Cloud사업팀</t>
+          <t>IDC운용팀</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2317,38 +2317,38 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>NTP-GROUP-03</t>
+          <t>NTP-GROUP-02</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>INCHEON IDC WLC</t>
+          <t>GWANGJU IDC Wireless-Bridge</t>
         </is>
       </c>
       <c r="Q20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R20" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>자동</t>
         </is>
       </c>
       <c r="T20" s="1" t="n">
-        <v>45669</v>
+        <v>45296</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ASSET0090</t>
+          <t>ASSET0072</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2358,17 +2358,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>보안부문</t>
+          <t>인프라부문</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>KT-WBR-SEOUL-20</t>
+          <t>KTBCP082</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>10.10.2.67</t>
+          <t>10.25.2.186</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Wireless-Bridge</t>
+          <t>WLC</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2388,22 +2388,22 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Cloud사업팀</t>
+          <t>IDC운용팀</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Network OS</t>
+          <t>Linux</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>IOS-XE</t>
+          <t>Rocky Linux</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2418,19 +2418,19 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>NTP-GROUP-01</t>
+          <t>NTP-GROUP-02</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>SEOUL IDC Wireless-Bridge</t>
+          <t>SEOUL IDC WLC</t>
         </is>
       </c>
       <c r="Q21" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="R21" s="1" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2438,13 +2438,13 @@
         </is>
       </c>
       <c r="T21" s="1" t="n">
-        <v>45414</v>
+        <v>45692</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ASSET0091</t>
+          <t>ASSET0097</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2454,17 +2454,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>인프라부문</t>
+          <t>네트워크부문</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>KT-AP-DAEJEON-21</t>
+          <t>KTAI039</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>10.10.5.193</t>
+          <t>10.24.1.249</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>WLC</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>NW운용1팀</t>
+          <t>NW운용2팀</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>적용</t>
+          <t>미적용</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2514,12 +2514,12 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>NTP-GROUP-02</t>
+          <t>NTP-GROUP-01</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>DAEJEON IDC AP</t>
+          <t>BUSAN IDC WLC</t>
         </is>
       </c>
       <c r="Q22" t="n">
@@ -2534,13 +2534,13 @@
         </is>
       </c>
       <c r="T22" s="1" t="n">
-        <v>45579</v>
+        <v>45881</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ASSET0092</t>
+          <t>ASSET0074</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2550,17 +2550,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>보안부문</t>
+          <t>인프라부문</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>KT-WLC-GWANGJU-22</t>
+          <t>KTIPTV025</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>10.10.8.24</t>
+          <t>10.22.1.140</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2570,12 +2570,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>WLC</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>운영</t>
+          <t>개발</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>적용</t>
+          <t>미적용</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2615,14 +2615,14 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>GWANGJU IDC WLC</t>
+          <t>SEOUL IDC AP</t>
         </is>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R23" s="1" t="n">
-        <v>46262</v>
+        <v>46257</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
@@ -2630,13 +2630,13 @@
         </is>
       </c>
       <c r="T23" s="1" t="n">
-        <v>45368</v>
+        <v>45303</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ASSET0093</t>
+          <t>ASSET0078</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2646,17 +2646,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>네트워크부문</t>
+          <t>인프라부문</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>KT-WLC-SEOUL-23</t>
+          <t>KTCLD031</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>10.10.7.4</t>
+          <t>10.20.1.212</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>IDC운용팀</t>
+          <t>NW운용1팀</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2686,12 +2686,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>JunOS</t>
+          <t>IOS-XE</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>13.4</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2711,14 +2711,14 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>SEOUL IDC WLC</t>
+          <t>GWANGJU IDC WLC</t>
         </is>
       </c>
       <c r="Q24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R24" s="1" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
@@ -2726,13 +2726,13 @@
         </is>
       </c>
       <c r="T24" s="1" t="n">
-        <v>46160</v>
+        <v>45920</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ASSET0094</t>
+          <t>ASSET0086</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2747,12 +2747,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KT-WBR-SEOUL-24</t>
+          <t>KTCLD039</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>10.10.5.57</t>
+          <t>10.20.2.2</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Wireless-Bridge</t>
+          <t>WLC</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2777,17 +2777,17 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Network OS</t>
+          <t>Linux</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>JunOS</t>
+          <t>Rocky Linux</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>15.9</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2802,12 +2802,12 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>NTP-GROUP-03</t>
+          <t>NTP-GROUP-01</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>SEOUL IDC Wireless-Bridge</t>
+          <t>GWANGJU IDC WLC</t>
         </is>
       </c>
       <c r="Q25" t="n">
@@ -2822,13 +2822,13 @@
         </is>
       </c>
       <c r="T25" s="1" t="n">
-        <v>45442</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ASSET0095</t>
+          <t>ASSET0096</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2838,17 +2838,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>네트워크부문</t>
+          <t>보안부문</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>KT-WLC-SEOUL-25</t>
+          <t>KTBCP022</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>10.10.4.62</t>
+          <t>10.25.1.107</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>WLC</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Cloud사업팀</t>
+          <t>NW운용1팀</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2898,19 +2898,19 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>NTP-GROUP-03</t>
+          <t>NTP-GROUP-02</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>SEOUL IDC WLC</t>
+          <t>BUSAN IDC AP</t>
         </is>
       </c>
       <c r="Q26" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R26" s="1" t="n">
-        <v>46260</v>
+        <v>46257</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
@@ -2918,13 +2918,13 @@
         </is>
       </c>
       <c r="T26" s="1" t="n">
-        <v>45733</v>
+        <v>45485</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ASSET0096</t>
+          <t>ASSET0073</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2934,17 +2934,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>보안부문</t>
+          <t>네트워크부문</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>KT-AP-BUSAN-26</t>
+          <t>KTAI064</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>10.10.13.129</t>
+          <t>10.24.2.129</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2959,12 +2959,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>운영</t>
+          <t>개발</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>NW운용1팀</t>
+          <t>Cloud사업팀</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>적용</t>
+          <t>미적용</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2999,14 +2999,14 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>BUSAN IDC AP</t>
+          <t>INCHEON IDC AP</t>
         </is>
       </c>
       <c r="Q27" t="n">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="R27" s="1" t="n">
-        <v>46257</v>
+        <v>46234</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
@@ -3014,13 +3014,13 @@
         </is>
       </c>
       <c r="T27" s="1" t="n">
-        <v>45485</v>
+        <v>45739</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ASSET0097</t>
+          <t>ASSET0079</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>KT-WLC-BUSAN-27</t>
+          <t>KTIPTV074</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>10.10.20.71</t>
+          <t>10.22.2.161</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>WLC</t>
+          <t>Wireless-Bridge</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>NW운용2팀</t>
+          <t>NW운용1팀</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -3080,7 +3080,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>미적용</t>
+          <t>적용</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3095,14 +3095,14 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>BUSAN IDC WLC</t>
+          <t>INCHEON IDC Wireless-Bridge</t>
         </is>
       </c>
       <c r="Q28" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R28" s="1" t="n">
-        <v>46257</v>
+        <v>46262</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
@@ -3110,13 +3110,13 @@
         </is>
       </c>
       <c r="T28" s="1" t="n">
-        <v>45881</v>
+        <v>45409</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASSET0098</t>
+          <t>ASSET0075</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3126,17 +3126,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>인프라부문</t>
+          <t>보안부문</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>KT-WLC-BUSAN-28</t>
+          <t>KTB-CP065</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>10.10.3.137</t>
+          <t>10.25.2.68</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>WLC</t>
+          <t>Wireless-Bridge</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3156,22 +3156,22 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Cloud사업팀</t>
+          <t>IDC운용팀</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Linux</t>
+          <t>Network OS</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Rocky Linux</t>
+          <t>PAN-OS</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3186,19 +3186,19 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>NTP-GROUP-03</t>
+          <t>NTP-GROUP-01</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>BUSAN IDC WLC</t>
+          <t>INCHEON IDC Wireless-Bridge</t>
         </is>
       </c>
       <c r="Q29" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="R29" s="1" t="n">
-        <v>46252</v>
+        <v>46261</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
@@ -3206,13 +3206,13 @@
         </is>
       </c>
       <c r="T29" s="1" t="n">
-        <v>45502</v>
+        <v>45840</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ASSET0099</t>
+          <t>ASSET0076</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3222,17 +3222,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>네트워크부문</t>
+          <t>인프라부문</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>KT-AP-BUSAN-29</t>
+          <t>KT-AP-GWANGJU-06</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>10.10.12.164</t>
+          <t>10.10.9.169</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Cloud사업팀</t>
+          <t>NW운용1팀</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -3282,19 +3282,19 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>NTP-GROUP-03</t>
+          <t>NTP-GROUP-01</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>BUSAN IDC AP</t>
+          <t>GWANGJU IDC AP</t>
         </is>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" s="1" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -3302,13 +3302,13 @@
         </is>
       </c>
       <c r="T30" s="1" t="n">
-        <v>45614</v>
+        <v>45581</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ASSET0100</t>
+          <t>ASSET0087</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3323,12 +3323,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>KT-WBR-SEOUL-30</t>
+          <t>KT-WBR-SEOUL-17</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>10.10.6.48</t>
+          <t>10.10.15.73</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3343,12 +3343,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>운영</t>
+          <t>개발</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>IDC운용팀</t>
+          <t>NW운용1팀</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3373,12 +3373,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>NTP-GROUP-01</t>
+          <t>NTP-GROUP-02</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3387,10 +3387,10 @@
         </is>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="R31" s="1" t="n">
-        <v>46262</v>
+        <v>46246</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
         </is>
       </c>
       <c r="T31" s="1" t="n">
-        <v>46070</v>
+        <v>46113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>